<commit_message>
chore: bundle weight-based sales import template (v1.0.61)
Frontend update: import template Excel now has unit/unitSize/saleStep
columns in the Блюда sheet, parser handles them, and the import UI
shows explicit weight-sales instructions.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/docs/шаблон-техкарты.xlsx
+++ b/frontend/docs/шаблон-техкарты.xlsx
@@ -122,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -148,6 +148,9 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="13" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -513,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:O71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -528,6 +531,9 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -591,6 +597,21 @@
           <t>Доступно</t>
         </is>
       </c>
+      <c r="M1" s="21" t="inlineStr">
+        <is>
+          <t>Ед. продажи</t>
+        </is>
+      </c>
+      <c r="N1" s="21" t="inlineStr">
+        <is>
+          <t>Размер порции (г)</t>
+        </is>
+      </c>
+      <c r="O1" s="21" t="inlineStr">
+        <is>
+          <t>Шаг (г)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -640,6 +661,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>100</v>
+      </c>
+      <c r="O2" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -689,6 +721,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -738,6 +781,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -787,6 +841,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -836,6 +901,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -883,6 +959,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -932,6 +1019,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -981,6 +1079,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1030,6 +1139,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1079,6 +1199,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1128,6 +1259,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1177,6 +1319,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1226,6 +1379,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1275,6 +1439,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1324,6 +1499,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1373,6 +1559,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1422,6 +1619,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1471,6 +1679,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1520,6 +1739,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>1</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1567,6 +1797,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>1</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1614,6 +1855,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1661,6 +1913,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>1</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1708,6 +1971,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>1</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1755,6 +2029,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>1</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1802,6 +2087,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1849,6 +2145,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1896,6 +2203,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>1</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1943,6 +2261,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>1</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1990,6 +2319,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N30" t="n">
+        <v>1</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2037,6 +2377,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>1</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2084,6 +2435,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>1</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2131,6 +2493,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>1</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2178,6 +2551,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N34" t="n">
+        <v>1</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -2227,6 +2611,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N35" t="n">
+        <v>1</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2274,6 +2669,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N36" t="n">
+        <v>1</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2321,6 +2727,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N37" t="n">
+        <v>1</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2368,6 +2785,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N38" t="n">
+        <v>1</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2415,6 +2843,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -2462,6 +2901,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
+        <v>1</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2509,6 +2959,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N41" t="n">
+        <v>1</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2556,6 +3017,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N42" t="n">
+        <v>1</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -2603,6 +3075,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
+        <v>1</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2650,6 +3133,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
+        <v>1</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2697,6 +3191,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>1</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2744,6 +3249,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>1</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2791,6 +3307,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
+        <v>1</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2838,6 +3365,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N48" t="n">
+        <v>1</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2885,6 +3423,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N49" t="n">
+        <v>1</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2932,6 +3481,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N50" t="n">
+        <v>1</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2979,6 +3539,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N51" t="n">
+        <v>1</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -3026,6 +3597,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N52" t="n">
+        <v>1</v>
+      </c>
+      <c r="O52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -3073,6 +3655,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
+        <v>1</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -3122,6 +3715,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N54" t="n">
+        <v>1</v>
+      </c>
+      <c r="O54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -3171,6 +3775,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N55" t="n">
+        <v>1</v>
+      </c>
+      <c r="O55" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -3220,6 +3835,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N56" t="n">
+        <v>1</v>
+      </c>
+      <c r="O56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -3269,6 +3895,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N57" t="n">
+        <v>1</v>
+      </c>
+      <c r="O57" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -3318,6 +3955,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N58" t="n">
+        <v>1</v>
+      </c>
+      <c r="O58" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -3365,6 +4013,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N59" t="n">
+        <v>1</v>
+      </c>
+      <c r="O59" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -3412,6 +4071,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N60" t="n">
+        <v>1</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -3459,6 +4129,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N61" t="n">
+        <v>1</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -3506,6 +4187,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N62" t="n">
+        <v>1</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -3553,6 +4245,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N63" t="n">
+        <v>1</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -3600,6 +4303,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N64" t="n">
+        <v>1</v>
+      </c>
+      <c r="O64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -3647,6 +4361,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N65" t="n">
+        <v>1</v>
+      </c>
+      <c r="O65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -3694,6 +4419,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N66" t="n">
+        <v>1</v>
+      </c>
+      <c r="O66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -3741,6 +4477,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N67" t="n">
+        <v>1</v>
+      </c>
+      <c r="O67" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -3788,6 +4535,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N68" t="n">
+        <v>1</v>
+      </c>
+      <c r="O68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -3835,6 +4593,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N69" t="n">
+        <v>1</v>
+      </c>
+      <c r="O69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -3882,6 +4651,17 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N70" t="n">
+        <v>1</v>
+      </c>
+      <c r="O70" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -3928,6 +4708,17 @@
         <is>
           <t>Да</t>
         </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="N71" t="n">
+        <v>1</v>
+      </c>
+      <c r="O71" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4209,7 +5000,6 @@
         <v>10.49</v>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -4580,7 +5370,6 @@
         <v>120.23</v>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -5005,7 +5794,6 @@
         <v>160.87</v>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
@@ -5430,7 +6218,6 @@
         <v>290.14</v>
       </c>
     </row>
-    <row r="59"/>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
@@ -5828,7 +6615,6 @@
         <v>279.16</v>
       </c>
     </row>
-    <row r="75"/>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
@@ -6167,7 +6953,6 @@
         <v>208.7</v>
       </c>
     </row>
-    <row r="89"/>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
@@ -6430,7 +7215,6 @@
         <v>251.2</v>
       </c>
     </row>
-    <row r="100"/>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
@@ -6612,7 +7396,6 @@
         <v>5.1</v>
       </c>
     </row>
-    <row r="108"/>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
@@ -6794,7 +7577,6 @@
         <v>6.7</v>
       </c>
     </row>
-    <row r="116"/>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
@@ -6976,7 +7758,6 @@
         <v>5.58</v>
       </c>
     </row>
-    <row r="124"/>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
@@ -7185,7 +7966,6 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="133"/>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
@@ -7529,7 +8309,6 @@
         <v>71</v>
       </c>
     </row>
-    <row r="147"/>
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
@@ -7900,7 +8679,6 @@
         <v>122.34</v>
       </c>
     </row>
-    <row r="162"/>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
         <is>
@@ -8109,7 +8887,6 @@
         <v>15.81</v>
       </c>
     </row>
-    <row r="171"/>
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
@@ -8318,7 +9095,6 @@
         <v>10.28</v>
       </c>
     </row>
-    <row r="180"/>
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
         <is>
@@ -8527,7 +9303,6 @@
         <v>61.64</v>
       </c>
     </row>
-    <row r="189"/>
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
         <is>
@@ -8736,7 +9511,6 @@
         <v>41.64</v>
       </c>
     </row>
-    <row r="198"/>
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
         <is>
@@ -8945,7 +9719,6 @@
         <v>40.74</v>
       </c>
     </row>
-    <row r="207"/>
     <row r="208">
       <c r="A208" s="3" t="inlineStr">
         <is>
@@ -9154,7 +9927,6 @@
         <v>46.64</v>
       </c>
     </row>
-    <row r="216"/>
     <row r="217">
       <c r="A217" s="3" t="inlineStr">
         <is>
@@ -9277,7 +10049,6 @@
         <v>137.06</v>
       </c>
     </row>
-    <row r="222"/>
     <row r="223">
       <c r="A223" s="3" t="inlineStr">
         <is>
@@ -9400,7 +10171,6 @@
         <v>147.06</v>
       </c>
     </row>
-    <row r="228"/>
     <row r="229">
       <c r="A229" s="3" t="inlineStr">
         <is>
@@ -9523,7 +10293,6 @@
         <v>122.06</v>
       </c>
     </row>
-    <row r="234"/>
     <row r="235">
       <c r="A235" s="3" t="inlineStr">
         <is>
@@ -9646,7 +10415,6 @@
         <v>122.06</v>
       </c>
     </row>
-    <row r="240"/>
     <row r="241">
       <c r="A241" s="3" t="inlineStr">
         <is>
@@ -9769,7 +10537,6 @@
         <v>77.06</v>
       </c>
     </row>
-    <row r="246"/>
     <row r="247">
       <c r="A247" s="3" t="inlineStr">
         <is>
@@ -9892,7 +10659,6 @@
         <v>122.06</v>
       </c>
     </row>
-    <row r="252"/>
     <row r="253">
       <c r="A253" s="3" t="inlineStr">
         <is>
@@ -10042,7 +10808,6 @@
         <v>135.74</v>
       </c>
     </row>
-    <row r="259"/>
     <row r="260">
       <c r="A260" s="3" t="inlineStr">
         <is>
@@ -10192,7 +10957,6 @@
         <v>139.06</v>
       </c>
     </row>
-    <row r="266"/>
     <row r="267">
       <c r="A267" s="3" t="inlineStr">
         <is>
@@ -10342,7 +11106,6 @@
         <v>149.06</v>
       </c>
     </row>
-    <row r="273"/>
     <row r="274">
       <c r="A274" s="3" t="inlineStr">
         <is>
@@ -10600,7 +11363,6 @@
         <v>20.29</v>
       </c>
     </row>
-    <row r="284"/>
     <row r="285">
       <c r="A285" s="3" t="inlineStr">
         <is>
@@ -11101,7 +11863,6 @@
         <v>231.54</v>
       </c>
     </row>
-    <row r="304"/>
     <row r="305">
       <c r="A305" s="3" t="inlineStr">
         <is>
@@ -11251,7 +12012,6 @@
         <v>53.56</v>
       </c>
     </row>
-    <row r="311"/>
     <row r="312">
       <c r="A312" s="3" t="inlineStr">
         <is>
@@ -11320,7 +12080,6 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="315"/>
     <row r="316">
       <c r="A316" s="3" t="inlineStr">
         <is>
@@ -11389,7 +12148,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="319"/>
     <row r="320">
       <c r="A320" s="3" t="inlineStr">
         <is>
@@ -11436,7 +12194,6 @@
         <v>10</v>
       </c>
     </row>
-    <row r="322"/>
     <row r="323">
       <c r="A323" s="3" t="inlineStr">
         <is>
@@ -11478,7 +12235,6 @@
         <v>10</v>
       </c>
     </row>
-    <row r="325"/>
     <row r="326">
       <c r="A326" s="3" t="inlineStr">
         <is>
@@ -11790,7 +12546,6 @@
         <v>14.15</v>
       </c>
     </row>
-    <row r="338"/>
     <row r="339">
       <c r="A339" s="3" t="inlineStr">
         <is>
@@ -12048,7 +12803,6 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="349"/>
     <row r="350">
       <c r="A350" s="3" t="inlineStr">
         <is>
@@ -12144,7 +12898,6 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="354"/>
     <row r="355">
       <c r="A355" s="3" t="inlineStr">
         <is>
@@ -12240,7 +12993,6 @@
         <v>1.71</v>
       </c>
     </row>
-    <row r="359"/>
     <row r="360">
       <c r="A360" s="3" t="inlineStr">
         <is>
@@ -12336,7 +13088,6 @@
         <v>2.76</v>
       </c>
     </row>
-    <row r="364"/>
     <row r="365">
       <c r="A365" s="3" t="inlineStr">
         <is>
@@ -12432,7 +13183,6 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="369"/>
     <row r="370">
       <c r="A370" s="3" t="inlineStr">
         <is>
@@ -12582,7 +13332,6 @@
         <v>5.1</v>
       </c>
     </row>
-    <row r="376"/>
     <row r="377">
       <c r="A377" s="3" t="inlineStr">
         <is>
@@ -12732,7 +13481,6 @@
         <v>4.6</v>
       </c>
     </row>
-    <row r="383"/>
     <row r="384">
       <c r="A384" s="3" t="inlineStr">
         <is>
@@ -12882,7 +13630,6 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="390"/>
     <row r="391">
       <c r="A391" s="3" t="inlineStr">
         <is>
@@ -13086,7 +13833,6 @@
         <v>16.63</v>
       </c>
     </row>
-    <row r="399"/>
     <row r="400">
       <c r="A400" s="3" t="inlineStr">
         <is>
@@ -13290,7 +14036,6 @@
         <v>13.77</v>
       </c>
     </row>
-    <row r="408"/>
     <row r="409">
       <c r="A409" s="3" t="inlineStr">
         <is>
@@ -13440,7 +14185,6 @@
         <v>13.72</v>
       </c>
     </row>
-    <row r="415"/>
     <row r="416">
       <c r="A416" s="3" t="inlineStr">
         <is>
@@ -13698,7 +14442,6 @@
         <v>131.88</v>
       </c>
     </row>
-    <row r="426"/>
     <row r="427">
       <c r="A427" s="3" t="inlineStr">
         <is>
@@ -13821,7 +14564,6 @@
         <v>100.49</v>
       </c>
     </row>
-    <row r="432"/>
     <row r="433">
       <c r="A433" s="3" t="inlineStr">
         <is>
@@ -13890,7 +14632,6 @@
         <v>16.27</v>
       </c>
     </row>
-    <row r="436"/>
     <row r="437">
       <c r="A437" s="3" t="inlineStr">
         <is>
@@ -14040,7 +14781,6 @@
         <v>16.25</v>
       </c>
     </row>
-    <row r="443"/>
     <row r="444">
       <c r="A444" s="3" t="inlineStr">
         <is>
@@ -14352,7 +15092,6 @@
         <v>757.4</v>
       </c>
     </row>
-    <row r="456"/>
     <row r="457">
       <c r="A457" s="3" t="inlineStr">
         <is>
@@ -14669,7 +15408,6 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="469"/>
     <row r="470">
       <c r="A470" s="3" t="inlineStr">
         <is>
@@ -14986,7 +15724,6 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="482"/>
     <row r="483">
       <c r="A483" s="3" t="inlineStr">
         <is>
@@ -15303,7 +16040,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="495"/>
     <row r="496">
       <c r="A496" s="3" t="inlineStr">
         <is>
@@ -15620,7 +16356,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="508"/>
     <row r="509">
       <c r="A509" s="3" t="inlineStr">
         <is>
@@ -15964,7 +16699,6 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="522"/>
     <row r="523">
       <c r="A523" s="3" t="inlineStr">
         <is>
@@ -16060,7 +16794,6 @@
         <v>19.29</v>
       </c>
     </row>
-    <row r="527"/>
     <row r="528">
       <c r="A528" s="3" t="inlineStr">
         <is>
@@ -16129,7 +16862,6 @@
         <v>19.89</v>
       </c>
     </row>
-    <row r="531"/>
     <row r="532">
       <c r="A532" s="3" t="inlineStr">
         <is>
@@ -16279,7 +17011,6 @@
         <v>13.09</v>
       </c>
     </row>
-    <row r="538"/>
     <row r="539">
       <c r="A539" s="3" t="inlineStr">
         <is>
@@ -16456,7 +17187,6 @@
         <v>20.16</v>
       </c>
     </row>
-    <row r="546"/>
     <row r="547">
       <c r="A547" s="3" t="inlineStr">
         <is>
@@ -16633,7 +17363,6 @@
         <v>30.76</v>
       </c>
     </row>
-    <row r="554"/>
     <row r="555">
       <c r="A555" s="3" t="inlineStr">
         <is>
@@ -16837,7 +17566,6 @@
         <v>43.14</v>
       </c>
     </row>
-    <row r="563"/>
     <row r="564">
       <c r="A564" s="3" t="inlineStr">
         <is>
@@ -17041,7 +17769,6 @@
         <v>36.73</v>
       </c>
     </row>
-    <row r="572"/>
     <row r="573">
       <c r="A573" s="3" t="inlineStr">
         <is>
@@ -17164,7 +17891,6 @@
         <v>131</v>
       </c>
     </row>
-    <row r="578"/>
     <row r="579">
       <c r="A579" s="3" t="inlineStr">
         <is>
@@ -17287,7 +18013,6 @@
         <v>131</v>
       </c>
     </row>
-    <row r="584"/>
     <row r="585">
       <c r="A585" s="3" t="inlineStr">
         <is>
@@ -17383,7 +18108,6 @@
         <v>24.64</v>
       </c>
     </row>
-    <row r="589"/>
     <row r="590">
       <c r="A590" s="3" t="inlineStr">
         <is>
@@ -17614,7 +18338,6 @@
         <v>28.67</v>
       </c>
     </row>
-    <row r="599"/>
     <row r="600">
       <c r="A600" s="3" t="inlineStr">
         <is>
@@ -17872,7 +18595,6 @@
         <v>34.47</v>
       </c>
     </row>
-    <row r="610"/>
     <row r="611">
       <c r="A611" s="3" t="inlineStr">
         <is>
@@ -22327,7 +23049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A71"/>
+  <dimension ref="A1:A97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -22607,6 +23329,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
@@ -22628,6 +23351,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
         <is>
@@ -22726,6 +23450,7 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
@@ -22747,6 +23472,7 @@
         </is>
       </c>
     </row>
+    <row r="66"/>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
@@ -22779,6 +23505,156 @@
       <c r="A71" t="inlineStr">
         <is>
           <t>5. Загрузите файл в RestOS → Настройки → Импорт</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>── НОВОЕ: Продажа по весу (граммы / килограммы) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Некоторые блюда (салаты, заготовки, сыры) удобно продавать по весу, а не порциями.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>В листе «Блюда» добавлены 3 новые колонки:</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Ед. продажи:    piece — штучно (шашлык, чай, кола) [по умолчанию]</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                    g     — за граммы (салат, сыр)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                    kg    — за килограмм</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Размер порции (г): для g — за сколько граммов указана цена (обычно 100).</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                       Для piece/kg — всегда 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Шаг (г):        минимальный шаг на весах (50 = округление до 50 г).</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                    0 = любой вес.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Примеры:</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Салат Каприз по 25 TJS за 100 г → Ед.=g, Размер=100, Шаг=50</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Сыр по 150 TJS за кг           → Ед.=kg, Размер=1, Шаг=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Шашлык по 80 TJS за порцию     → Ед.=piece, Размер=1, Шаг=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Цена в колонке G указывается ЗА ЕДИНИЦУ ПРОДАЖИ:</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Для piece — за 1 штуку</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Для g     — за 100 г (или сколько указано в «Размер порции»)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Для kg    — за 1 кг</t>
         </is>
       </c>
     </row>

</xml_diff>